<commit_message>
Update House PTR data (2026-09-06)
</commit_message>
<xml_diff>
--- a/data/03_verification/House_PTR_Verification_2026.xlsx
+++ b/data/03_verification/House_PTR_Verification_2026.xlsx
@@ -9,8 +9,7 @@
   <sheets>
     <sheet name="House XML Index" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Verification" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Missing PTRs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Parser Flagged" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Parser Flagged" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +28,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -39,11 +38,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,10 +53,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6218,57 +6211,61 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="inlineStr">
+      <c r="A135" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B135" s="2" t="inlineStr">
+      <c r="B135" s="1" t="inlineStr">
         <is>
           <t>Beyer</t>
         </is>
       </c>
-      <c r="C135" s="2" t="inlineStr">
+      <c r="C135" s="1" t="inlineStr">
         <is>
           <t>Donald Sternoff</t>
         </is>
       </c>
-      <c r="D135" s="2" t="inlineStr">
+      <c r="D135" s="1" t="inlineStr">
         <is>
           <t>Jr</t>
         </is>
       </c>
-      <c r="E135" s="2" t="inlineStr">
+      <c r="E135" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F135" s="2" t="inlineStr">
+      <c r="F135" s="1" t="inlineStr">
         <is>
           <t>VA08</t>
         </is>
       </c>
-      <c r="G135" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H135" s="2" t="inlineStr">
+      <c r="G135" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H135" s="1" t="inlineStr">
         <is>
           <t>9/1/2026</t>
         </is>
       </c>
-      <c r="I135" s="2" t="inlineStr">
+      <c r="I135" s="1" t="inlineStr">
         <is>
           <t>20035349</t>
         </is>
       </c>
-      <c r="J135" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K135" s="2" t="inlineStr"/>
+      <c r="J135" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K135" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr"/>
@@ -13242,53 +13239,57 @@
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="2" t="inlineStr">
+      <c r="A295" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B295" s="2" t="inlineStr">
+      <c r="B295" s="1" t="inlineStr">
         <is>
           <t>Cohen</t>
         </is>
       </c>
-      <c r="C295" s="2" t="inlineStr">
+      <c r="C295" s="1" t="inlineStr">
         <is>
           <t>Steve</t>
         </is>
       </c>
-      <c r="D295" s="2" t="inlineStr"/>
-      <c r="E295" s="2" t="inlineStr">
+      <c r="D295" s="1" t="inlineStr"/>
+      <c r="E295" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F295" s="2" t="inlineStr">
+      <c r="F295" s="1" t="inlineStr">
         <is>
           <t>TN09</t>
         </is>
       </c>
-      <c r="G295" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H295" s="2" t="inlineStr">
+      <c r="G295" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H295" s="1" t="inlineStr">
         <is>
           <t>9/1/2026</t>
         </is>
       </c>
-      <c r="I295" s="2" t="inlineStr">
+      <c r="I295" s="1" t="inlineStr">
         <is>
           <t>20035350</t>
         </is>
       </c>
-      <c r="J295" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K295" s="2" t="inlineStr"/>
+      <c r="J295" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K295" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="1" t="inlineStr">
@@ -21986,49 +21987,53 @@
       </c>
     </row>
     <row r="491">
-      <c r="A491" s="2" t="inlineStr"/>
-      <c r="B491" s="2" t="inlineStr">
+      <c r="A491" s="1" t="inlineStr"/>
+      <c r="B491" s="1" t="inlineStr">
         <is>
           <t>Fields</t>
         </is>
       </c>
-      <c r="C491" s="2" t="inlineStr">
+      <c r="C491" s="1" t="inlineStr">
         <is>
           <t>Cleo</t>
         </is>
       </c>
-      <c r="D491" s="2" t="inlineStr"/>
-      <c r="E491" s="2" t="inlineStr">
+      <c r="D491" s="1" t="inlineStr"/>
+      <c r="E491" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F491" s="2" t="inlineStr">
+      <c r="F491" s="1" t="inlineStr">
         <is>
           <t>LA06</t>
         </is>
       </c>
-      <c r="G491" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H491" s="2" t="inlineStr">
+      <c r="G491" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H491" s="1" t="inlineStr">
         <is>
           <t>9/2/2026</t>
         </is>
       </c>
-      <c r="I491" s="2" t="inlineStr">
+      <c r="I491" s="1" t="inlineStr">
         <is>
           <t>20035345</t>
         </is>
       </c>
-      <c r="J491" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K491" s="2" t="inlineStr"/>
+      <c r="J491" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K491" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr"/>
@@ -30404,53 +30409,57 @@
       </c>
     </row>
     <row r="681">
-      <c r="A681" s="2" t="inlineStr">
+      <c r="A681" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B681" s="2" t="inlineStr">
+      <c r="B681" s="1" t="inlineStr">
         <is>
           <t>Hern</t>
         </is>
       </c>
-      <c r="C681" s="2" t="inlineStr">
+      <c r="C681" s="1" t="inlineStr">
         <is>
           <t>Kevin</t>
         </is>
       </c>
-      <c r="D681" s="2" t="inlineStr"/>
-      <c r="E681" s="2" t="inlineStr">
+      <c r="D681" s="1" t="inlineStr"/>
+      <c r="E681" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F681" s="2" t="inlineStr">
+      <c r="F681" s="1" t="inlineStr">
         <is>
           <t>OK01</t>
         </is>
       </c>
-      <c r="G681" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H681" s="2" t="inlineStr">
+      <c r="G681" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H681" s="1" t="inlineStr">
         <is>
           <t>9/1/2026</t>
         </is>
       </c>
-      <c r="I681" s="2" t="inlineStr">
+      <c r="I681" s="1" t="inlineStr">
         <is>
           <t>20035326</t>
         </is>
       </c>
-      <c r="J681" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K681" s="2" t="inlineStr"/>
+      <c r="J681" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K681" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="682">
       <c r="A682" t="inlineStr"/>
@@ -33201,53 +33210,57 @@
       </c>
     </row>
     <row r="746">
-      <c r="A746" s="2" t="inlineStr">
+      <c r="A746" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B746" s="2" t="inlineStr">
+      <c r="B746" s="1" t="inlineStr">
         <is>
           <t>Jackson</t>
         </is>
       </c>
-      <c r="C746" s="2" t="inlineStr">
+      <c r="C746" s="1" t="inlineStr">
         <is>
           <t>Jonathan</t>
         </is>
       </c>
-      <c r="D746" s="2" t="inlineStr"/>
-      <c r="E746" s="2" t="inlineStr">
+      <c r="D746" s="1" t="inlineStr"/>
+      <c r="E746" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F746" s="2" t="inlineStr">
+      <c r="F746" s="1" t="inlineStr">
         <is>
           <t>IL01</t>
         </is>
       </c>
-      <c r="G746" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H746" s="2" t="inlineStr">
+      <c r="G746" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H746" s="1" t="inlineStr">
         <is>
           <t>9/3/2026</t>
         </is>
       </c>
-      <c r="I746" s="2" t="inlineStr">
+      <c r="I746" s="1" t="inlineStr">
         <is>
           <t>20035370</t>
         </is>
       </c>
-      <c r="J746" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K746" s="2" t="inlineStr"/>
+      <c r="J746" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K746" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="747">
       <c r="A747" t="inlineStr">
@@ -36198,53 +36211,57 @@
       </c>
     </row>
     <row r="811">
-      <c r="A811" s="2" t="inlineStr">
+      <c r="A811" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B811" s="2" t="inlineStr">
+      <c r="B811" s="1" t="inlineStr">
         <is>
           <t>Keating</t>
         </is>
       </c>
-      <c r="C811" s="2" t="inlineStr">
+      <c r="C811" s="1" t="inlineStr">
         <is>
           <t>William R.</t>
         </is>
       </c>
-      <c r="D811" s="2" t="inlineStr"/>
-      <c r="E811" s="2" t="inlineStr">
+      <c r="D811" s="1" t="inlineStr"/>
+      <c r="E811" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F811" s="2" t="inlineStr">
+      <c r="F811" s="1" t="inlineStr">
         <is>
           <t>MA09</t>
         </is>
       </c>
-      <c r="G811" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H811" s="2" t="inlineStr">
+      <c r="G811" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H811" s="1" t="inlineStr">
         <is>
           <t>8/25/2026</t>
         </is>
       </c>
-      <c r="I811" s="2" t="inlineStr">
+      <c r="I811" s="1" t="inlineStr">
         <is>
           <t>20035293</t>
         </is>
       </c>
-      <c r="J811" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K811" s="2" t="inlineStr"/>
+      <c r="J811" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K811" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="812">
       <c r="A812" t="inlineStr"/>
@@ -44832,57 +44849,61 @@
       </c>
     </row>
     <row r="1005">
-      <c r="A1005" s="2" t="inlineStr">
+      <c r="A1005" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B1005" s="2" t="inlineStr">
+      <c r="B1005" s="1" t="inlineStr">
         <is>
           <t>McGuire</t>
         </is>
       </c>
-      <c r="C1005" s="2" t="inlineStr">
+      <c r="C1005" s="1" t="inlineStr">
         <is>
           <t>John J Mr</t>
         </is>
       </c>
-      <c r="D1005" s="2" t="inlineStr">
+      <c r="D1005" s="1" t="inlineStr">
         <is>
           <t>III</t>
         </is>
       </c>
-      <c r="E1005" s="2" t="inlineStr">
+      <c r="E1005" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F1005" s="2" t="inlineStr">
+      <c r="F1005" s="1" t="inlineStr">
         <is>
           <t>VA05</t>
         </is>
       </c>
-      <c r="G1005" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H1005" s="2" t="inlineStr">
+      <c r="G1005" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H1005" s="1" t="inlineStr">
         <is>
           <t>9/2/2026</t>
         </is>
       </c>
-      <c r="I1005" s="2" t="inlineStr">
+      <c r="I1005" s="1" t="inlineStr">
         <is>
           <t>20035367</t>
         </is>
       </c>
-      <c r="J1005" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K1005" s="2" t="inlineStr"/>
+      <c r="J1005" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K1005" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="1006">
       <c r="A1006" t="inlineStr"/>
@@ -48695,53 +48716,57 @@
       </c>
     </row>
     <row r="1088">
-      <c r="A1088" s="2" t="inlineStr">
+      <c r="A1088" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B1088" s="2" t="inlineStr">
+      <c r="B1088" s="1" t="inlineStr">
         <is>
           <t>Morrison</t>
         </is>
       </c>
-      <c r="C1088" s="2" t="inlineStr">
+      <c r="C1088" s="1" t="inlineStr">
         <is>
           <t>Kelly Louise</t>
         </is>
       </c>
-      <c r="D1088" s="2" t="inlineStr"/>
-      <c r="E1088" s="2" t="inlineStr">
+      <c r="D1088" s="1" t="inlineStr"/>
+      <c r="E1088" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F1088" s="2" t="inlineStr">
+      <c r="F1088" s="1" t="inlineStr">
         <is>
           <t>MN03</t>
         </is>
       </c>
-      <c r="G1088" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H1088" s="2" t="inlineStr">
+      <c r="G1088" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H1088" s="1" t="inlineStr">
         <is>
           <t>8/25/2026</t>
         </is>
       </c>
-      <c r="I1088" s="2" t="inlineStr">
+      <c r="I1088" s="1" t="inlineStr">
         <is>
           <t>20035244</t>
         </is>
       </c>
-      <c r="J1088" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K1088" s="2" t="inlineStr"/>
+      <c r="J1088" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K1088" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="1089">
       <c r="A1089" t="inlineStr"/>
@@ -49173,53 +49198,57 @@
       </c>
     </row>
     <row r="1098">
-      <c r="A1098" s="2" t="inlineStr">
+      <c r="A1098" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B1098" s="2" t="inlineStr">
+      <c r="B1098" s="1" t="inlineStr">
         <is>
           <t>Moskowitz</t>
         </is>
       </c>
-      <c r="C1098" s="2" t="inlineStr">
+      <c r="C1098" s="1" t="inlineStr">
         <is>
           <t>Jared</t>
         </is>
       </c>
-      <c r="D1098" s="2" t="inlineStr"/>
-      <c r="E1098" s="2" t="inlineStr">
+      <c r="D1098" s="1" t="inlineStr"/>
+      <c r="E1098" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F1098" s="2" t="inlineStr">
+      <c r="F1098" s="1" t="inlineStr">
         <is>
           <t>FL23</t>
         </is>
       </c>
-      <c r="G1098" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H1098" s="2" t="inlineStr">
+      <c r="G1098" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H1098" s="1" t="inlineStr">
         <is>
           <t>8/27/2026</t>
         </is>
       </c>
-      <c r="I1098" s="2" t="inlineStr">
+      <c r="I1098" s="1" t="inlineStr">
         <is>
           <t>20035243</t>
         </is>
       </c>
-      <c r="J1098" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K1098" s="2" t="inlineStr"/>
+      <c r="J1098" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K1098" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="1099">
       <c r="A1099" t="inlineStr"/>
@@ -57861,102 +57890,110 @@
       </c>
     </row>
     <row r="1298">
-      <c r="A1298" s="2" t="inlineStr">
+      <c r="A1298" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B1298" s="2" t="inlineStr">
+      <c r="B1298" s="1" t="inlineStr">
         <is>
           <t>Rulli</t>
         </is>
       </c>
-      <c r="C1298" s="2" t="inlineStr">
+      <c r="C1298" s="1" t="inlineStr">
         <is>
           <t>Michael</t>
         </is>
       </c>
-      <c r="D1298" s="2" t="inlineStr"/>
-      <c r="E1298" s="2" t="inlineStr">
+      <c r="D1298" s="1" t="inlineStr"/>
+      <c r="E1298" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F1298" s="2" t="inlineStr">
+      <c r="F1298" s="1" t="inlineStr">
         <is>
           <t>OH06</t>
         </is>
       </c>
-      <c r="G1298" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H1298" s="2" t="inlineStr">
+      <c r="G1298" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H1298" s="1" t="inlineStr">
         <is>
           <t>8/25/2026</t>
         </is>
       </c>
-      <c r="I1298" s="2" t="inlineStr">
+      <c r="I1298" s="1" t="inlineStr">
         <is>
           <t>20035309</t>
         </is>
       </c>
-      <c r="J1298" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K1298" s="2" t="inlineStr"/>
+      <c r="J1298" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K1298" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="1299">
-      <c r="A1299" s="2" t="inlineStr">
+      <c r="A1299" s="1" t="inlineStr">
         <is>
           <t>Hon.</t>
         </is>
       </c>
-      <c r="B1299" s="2" t="inlineStr">
+      <c r="B1299" s="1" t="inlineStr">
         <is>
           <t>Rulli</t>
         </is>
       </c>
-      <c r="C1299" s="2" t="inlineStr">
+      <c r="C1299" s="1" t="inlineStr">
         <is>
           <t>Michael</t>
         </is>
       </c>
-      <c r="D1299" s="2" t="inlineStr"/>
-      <c r="E1299" s="2" t="inlineStr">
+      <c r="D1299" s="1" t="inlineStr"/>
+      <c r="E1299" s="1" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="F1299" s="2" t="inlineStr">
+      <c r="F1299" s="1" t="inlineStr">
         <is>
           <t>OH06</t>
         </is>
       </c>
-      <c r="G1299" s="2" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="H1299" s="2" t="inlineStr">
+      <c r="G1299" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="H1299" s="1" t="inlineStr">
         <is>
           <t>9/2/2026</t>
         </is>
       </c>
-      <c r="I1299" s="2" t="inlineStr">
+      <c r="I1299" s="1" t="inlineStr">
         <is>
           <t>20035365</t>
         </is>
       </c>
-      <c r="J1299" s="2" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="K1299" s="2" t="inlineStr"/>
+      <c r="J1299" s="1" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="K1299" s="1" t="inlineStr">
+        <is>
+          <t>not_yet_parsed</t>
+        </is>
+      </c>
     </row>
     <row r="1300">
       <c r="A1300" t="inlineStr"/>
@@ -70899,7 +70936,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>364</v>
+        <v>375</v>
       </c>
     </row>
     <row r="5">
@@ -70909,7 +70946,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>364</v>
+        <v>375</v>
       </c>
     </row>
     <row r="6">
@@ -70919,7 +70956,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -70949,7 +70986,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -70960,7 +70997,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -70975,104 +71012,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Missing DocID</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>20035243</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>20035244</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>20035293</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>20035309</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>20035326</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>20035345</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>20035349</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>20035350</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>20035365</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>20035367</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>20035370</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:A44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Update House PTR data (2026-09-12)
</commit_message>
<xml_diff>
--- a/data/03_verification/House_PTR_Verification_2026.xlsx
+++ b/data/03_verification/House_PTR_Verification_2026.xlsx
@@ -12351,7 +12351,7 @@
       </c>
       <c r="K275" s="1" t="inlineStr">
         <is>
-          <t>not_yet_parsed</t>
+          <t>geometry_v8</t>
         </is>
       </c>
     </row>
@@ -72147,7 +72147,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">

</xml_diff>